<commit_message>
Exclude Digital Inspections cases from Custom Roles QA workbook (176 cases)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/CustomRoles_TestSuite_QA_Report.xlsx
+++ b/CustomRoles_TestSuite_QA_Report.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -614,59 +614,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Digital Inspections</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>121</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>98</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>297</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F6" s="4" t="n">
+      <c r="B5" s="4" t="n">
+        <v>176</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>137</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>We ran the full Custom Roles test suite: 297 tests in total. 235 passed, 5 failed, 50 could not be completed (blocked), and 7 turned out not to apply to this build. The 'Failed Tests' tab has full step-by-step instructions to reproduce each problem; the 'Blocked Tests' tab explains why each blocked test could not be run and what is needed to run it. Blocked tests were re-tried on disposable test data where possible before being counted here.</t>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>We ran the Custom Roles test suite: 176 tests in total (Digital Inspections cases excluded per request). 137 passed, 3 failed, 29 could not be completed (blocked), and 7 turned out not to apply to this build. The 'Failed Tests' tab has full step-by-step instructions to reproduce each problem; the 'Blocked Tests' tab explains why each blocked test could not be run and what is needed to run it. Blocked tests were re-tried on disposable test data where possible before being counted here.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -678,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F236"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5130,3301 +5108,6 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="120" customHeight="1">
-      <c r="A139" s="6" t="inlineStr">
-        <is>
-          <t>DI-001</t>
-        </is>
-      </c>
-      <c r="B139" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C139" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E139" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit, has Delete) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F139" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="135" customHeight="1">
-      <c r="A140" s="6" t="inlineStr">
-        <is>
-          <t>DI-002</t>
-        </is>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>Administrator - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="120" customHeight="1">
-      <c r="A141" s="6" t="inlineStr">
-        <is>
-          <t>DI-004</t>
-        </is>
-      </c>
-      <c r="B141" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C141" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E141" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F141" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="90" customHeight="1">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>DI-007</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>Administrator - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="120" customHeight="1">
-      <c r="A143" s="6" t="inlineStr">
-        <is>
-          <t>DI-008</t>
-        </is>
-      </c>
-      <c r="B143" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C143" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - Are you sure you want to remove this inspection?" (Cancel / Remove).
-Step 4: On Remove, the inspection is removed from the line.
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on an in-progress inspection (removal gated by this permission). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F143" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="135" customHeight="1">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>DI-009</t>
-        </is>
-      </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t>Administrator - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - This inspection has a generated PDF report. Are you sure you want to remove it?" (Cancel / Remove).
-Step 4: On Remove, the completed inspection is removed.
-Build note: removal may require the work order line to NOT be marked complete (mark line Uncomplete first).
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on a completed inspection (with PDF). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="120" customHeight="1">
-      <c r="A145" s="6" t="inlineStr">
-        <is>
-          <t>DI-010</t>
-        </is>
-      </c>
-      <c r="B145" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C145" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The completed inspection reopens for editing via the Open control.
-Step 4: VIU - confirm reopen behavior for an inspection already submitted with a generated PDF report (open question from build testing).
-Spec reference: SV-7509 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E145" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the Open/Reopen control on a completed inspection is available (reopen gated by this permission). Actual reopen not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F145" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="120" customHeight="1">
-      <c r="A146" s="6" t="inlineStr">
-        <is>
-          <t>DI-011</t>
-        </is>
-      </c>
-      <c r="B146" s="2" t="inlineStr">
-        <is>
-          <t>Administrator - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Settings &gt; Service is accessible.
-Step 3: The Inspection Templates section is available.
-Step 4: A new template can be created with fields: Checklist, Short Text, Long Text, Measurements, Photo, Instructions.
-Spec reference: SV-7521 · Digital Inspections — Administrator role</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>Settings &gt; Service is accessible and the Service section exposes "Inspection Templates" (verified in Tech UI: SERVICE menu group shown, page loads with template list + "New/Create" control). A template can be created with the listed field types.</t>
-        </is>
-      </c>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role has both. Verified live in Tech UI. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="120" customHeight="1">
-      <c r="A147" s="6" t="inlineStr">
-        <is>
-          <t>DI-012</t>
-        </is>
-      </c>
-      <c r="B147" s="3" t="inlineStr">
-        <is>
-          <t>Service Manager - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C147" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D147" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E147" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit, has Delete) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F147" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="135" customHeight="1">
-      <c r="A148" s="6" t="inlineStr">
-        <is>
-          <t>DI-013</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="120" customHeight="1">
-      <c r="A149" s="6" t="inlineStr">
-        <is>
-          <t>DI-015</t>
-        </is>
-      </c>
-      <c r="B149" s="3" t="inlineStr">
-        <is>
-          <t>Service Manager - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C149" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E149" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="90" customHeight="1">
-      <c r="A150" s="6" t="inlineStr">
-        <is>
-          <t>DI-018</t>
-        </is>
-      </c>
-      <c r="B150" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="120" customHeight="1">
-      <c r="A151" s="6" t="inlineStr">
-        <is>
-          <t>DI-019</t>
-        </is>
-      </c>
-      <c r="B151" s="3" t="inlineStr">
-        <is>
-          <t>Service Manager - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C151" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D151" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - Are you sure you want to remove this inspection?" (Cancel / Remove).
-Step 4: On Remove, the inspection is removed from the line.
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E151" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on an in-progress inspection (removal gated by this permission). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F151" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="135" customHeight="1">
-      <c r="A152" s="6" t="inlineStr">
-        <is>
-          <t>DI-020</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - This inspection has a generated PDF report. Are you sure you want to remove it?" (Cancel / Remove).
-Step 4: On Remove, the completed inspection is removed.
-Build note: removal may require the work order line to NOT be marked complete (mark line Uncomplete first).
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on a completed inspection (with PDF). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="120" customHeight="1">
-      <c r="A153" s="6" t="inlineStr">
-        <is>
-          <t>DI-021</t>
-        </is>
-      </c>
-      <c r="B153" s="3" t="inlineStr">
-        <is>
-          <t>Service Manager - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C153" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D153" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The completed inspection reopens for editing via the Open control.
-Step 4: VIU - confirm reopen behavior for an inspection already submitted with a generated PDF report (open question from build testing).
-Spec reference: SV-7509 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E153" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the Open/Reopen control on a completed inspection is available (reopen gated by this permission). Actual reopen not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F153" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="255" customHeight="1">
-      <c r="A154" s="6" t="inlineStr">
-        <is>
-          <t>DI-022</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Service Manager role</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="120" customHeight="1">
-      <c r="A155" s="6" t="inlineStr">
-        <is>
-          <t>DI-023</t>
-        </is>
-      </c>
-      <c r="B155" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C155" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D155" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E155" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit, has Delete) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F155" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="135" customHeight="1">
-      <c r="A156" s="6" t="inlineStr">
-        <is>
-          <t>DI-024</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C156" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D156" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E156" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F156" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="120" customHeight="1">
-      <c r="A157" s="6" t="inlineStr">
-        <is>
-          <t>DI-026</t>
-        </is>
-      </c>
-      <c r="B157" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C157" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D157" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E157" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F157" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="90" customHeight="1">
-      <c r="A158" s="6" t="inlineStr">
-        <is>
-          <t>DI-029</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" ht="120" customHeight="1">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>DI-030</t>
-        </is>
-      </c>
-      <c r="B159" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C159" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D159" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - Are you sure you want to remove this inspection?" (Cancel / Remove).
-Step 4: On Remove, the inspection is removed from the line.
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E159" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on an in-progress inspection (removal gated by this permission). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F159" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="135" customHeight="1">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t>DI-031</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - This inspection has a generated PDF report. Are you sure you want to remove it?" (Cancel / Remove).
-Step 4: On Remove, the completed inspection is removed.
-Build note: removal may require the work order line to NOT be marked complete (mark line Uncomplete first).
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on a completed inspection (with PDF). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="120" customHeight="1">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>DI-032</t>
-        </is>
-      </c>
-      <c r="B161" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C161" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D161" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The completed inspection reopens for editing via the Open control.
-Step 4: VIU - confirm reopen behavior for an inspection already submitted with a generated PDF report (open question from build testing).
-Spec reference: SV-7509 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E161" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the Open/Reopen control on a completed inspection is available (reopen gated by this permission). Actual reopen not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F161" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162" ht="255" customHeight="1">
-      <c r="A162" s="6" t="inlineStr">
-        <is>
-          <t>DI-033</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Senior Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="163" ht="120" customHeight="1">
-      <c r="A163" s="6" t="inlineStr">
-        <is>
-          <t>DI-034</t>
-        </is>
-      </c>
-      <c r="B163" s="3" t="inlineStr">
-        <is>
-          <t>Service Advisor - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C163" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D163" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E163" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit, has Delete) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F163" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="164" ht="135" customHeight="1">
-      <c r="A164" s="6" t="inlineStr">
-        <is>
-          <t>DI-035</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="165" ht="120" customHeight="1">
-      <c r="A165" s="6" t="inlineStr">
-        <is>
-          <t>DI-037</t>
-        </is>
-      </c>
-      <c r="B165" s="3" t="inlineStr">
-        <is>
-          <t>Service Advisor - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C165" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D165" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E165" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F165" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" ht="90" customHeight="1">
-      <c r="A166" s="6" t="inlineStr">
-        <is>
-          <t>DI-040</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="167" ht="120" customHeight="1">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>DI-041</t>
-        </is>
-      </c>
-      <c r="B167" s="3" t="inlineStr">
-        <is>
-          <t>Service Advisor - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C167" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D167" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - Are you sure you want to remove this inspection?" (Cancel / Remove).
-Step 4: On Remove, the inspection is removed from the line.
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E167" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on an in-progress inspection (removal gated by this permission). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F167" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="168" ht="135" customHeight="1">
-      <c r="A168" s="6" t="inlineStr">
-        <is>
-          <t>DI-042</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - This inspection has a generated PDF report. Are you sure you want to remove it?" (Cancel / Remove).
-Step 4: On Remove, the completed inspection is removed.
-Build note: removal may require the work order line to NOT be marked complete (mark line Uncomplete first).
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on a completed inspection (with PDF). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169" ht="120" customHeight="1">
-      <c r="A169" s="6" t="inlineStr">
-        <is>
-          <t>DI-043</t>
-        </is>
-      </c>
-      <c r="B169" s="3" t="inlineStr">
-        <is>
-          <t>Service Advisor - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C169" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D169" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The completed inspection reopens for editing via the Open control.
-Step 4: VIU - confirm reopen behavior for an inspection already submitted with a generated PDF report (open question from build testing).
-Spec reference: SV-7509 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E169" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the Open/Reopen control on a completed inspection is available (reopen gated by this permission). Actual reopen not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F169" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" ht="255" customHeight="1">
-      <c r="A170" s="6" t="inlineStr">
-        <is>
-          <t>DI-044</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Service Advisor role</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="171" ht="105" customHeight="1">
-      <c r="A171" s="6" t="inlineStr">
-        <is>
-          <t>DI-045</t>
-        </is>
-      </c>
-      <c r="B171" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C171" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D171" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E171" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit, has Delete) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F171" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172" ht="135" customHeight="1">
-      <c r="A172" s="6" t="inlineStr">
-        <is>
-          <t>DI-046</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>Foreman - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E172" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="173" ht="120" customHeight="1">
-      <c r="A173" s="6" t="inlineStr">
-        <is>
-          <t>DI-048</t>
-        </is>
-      </c>
-      <c r="B173" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C173" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F173" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174" ht="90" customHeight="1">
-      <c r="A174" s="6" t="inlineStr">
-        <is>
-          <t>DI-051</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>Foreman - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E174" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="175" ht="120" customHeight="1">
-      <c r="A175" s="6" t="inlineStr">
-        <is>
-          <t>DI-052</t>
-        </is>
-      </c>
-      <c r="B175" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C175" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D175" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - Are you sure you want to remove this inspection?" (Cancel / Remove).
-Step 4: On Remove, the inspection is removed from the line.
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E175" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on an in-progress inspection (removal gated by this permission). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F175" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176" ht="120" customHeight="1">
-      <c r="A176" s="6" t="inlineStr">
-        <is>
-          <t>DI-053</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>Foreman - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: A confirmation dialog appears: "Remove inspection - This inspection has a generated PDF report. Are you sure you want to remove it?" (Cancel / Remove).
-Step 4: On Remove, the completed inspection is removed.
-Build note: removal may require the work order line to NOT be marked complete (mark line Uncomplete first).
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the remove (bin) control is available on a completed inspection (with PDF). Actual destructive removal not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="177" ht="120" customHeight="1">
-      <c r="A177" s="6" t="inlineStr">
-        <is>
-          <t>DI-054</t>
-        </is>
-      </c>
-      <c r="B177" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C177" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D177" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The completed inspection reopens for editing via the Open control.
-Step 4: VIU - confirm reopen behavior for an inspection already submitted with a generated PDF report (open question from build testing).
-Spec reference: SV-7509 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesDelete -&gt; the Open/Reopen control on a completed inspection is available (reopen gated by this permission). Actual reopen not executed on shared staging.</t>
-        </is>
-      </c>
-      <c r="F177" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178" ht="255" customHeight="1">
-      <c r="A178" s="6" t="inlineStr">
-        <is>
-          <t>DI-055</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>Foreman - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Foreman role</t>
-        </is>
-      </c>
-      <c r="E178" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179" ht="105" customHeight="1">
-      <c r="A179" s="6" t="inlineStr">
-        <is>
-          <t>DI-056</t>
-        </is>
-      </c>
-      <c r="B179" s="3" t="inlineStr">
-        <is>
-          <t>Technician - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C179" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D179" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E179" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F179" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180" ht="135" customHeight="1">
-      <c r="A180" s="6" t="inlineStr">
-        <is>
-          <t>DI-057</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Technician - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: On a NEW line the technician is creating, the inspection is added and "Inspection added to line." is shown.
-Step 5: VIU - on an existing/approved line (read-only under Tech View) adding may be blocked; confirm intended behavior.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E180" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="181" ht="120" customHeight="1">
-      <c r="A181" s="6" t="inlineStr">
-        <is>
-          <t>DI-059</t>
-        </is>
-      </c>
-      <c r="B181" s="3" t="inlineStr">
-        <is>
-          <t>Technician - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C181" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: The technician can fill/edit inspection items on a NEW line, or on an existing line only if that line is NOT marked complete (read-only once the line is completed).
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F181" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="182" ht="90" customHeight="1">
-      <c r="A182" s="6" t="inlineStr">
-        <is>
-          <t>DI-062</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>Technician - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="183" ht="120" customHeight="1">
-      <c r="A183" s="6" t="inlineStr">
-        <is>
-          <t>DI-063</t>
-        </is>
-      </c>
-      <c r="B183" s="3" t="inlineStr">
-        <is>
-          <t>Technician - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C183" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D183" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing an inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E183" s="3" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available - role lacks workOrderLinesDelete (Work Order Lines: Delete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F183" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="184" ht="120" customHeight="1">
-      <c r="A184" s="6" t="inlineStr">
-        <is>
-          <t>DI-064</t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="inlineStr">
-        <is>
-          <t>Technician - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C184" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available for a completed inspection - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F184" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="185" ht="120" customHeight="1">
-      <c r="A185" s="6" t="inlineStr">
-        <is>
-          <t>DI-065</t>
-        </is>
-      </c>
-      <c r="B185" s="3" t="inlineStr">
-        <is>
-          <t>Technician - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C185" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D185" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Reopen is NOT available - reopening a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E185" s="3" t="inlineStr">
-        <is>
-          <t>Reopen is NOT available - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F185" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="186" ht="255" customHeight="1">
-      <c r="A186" s="6" t="inlineStr">
-        <is>
-          <t>DI-066</t>
-        </is>
-      </c>
-      <c r="B186" s="2" t="inlineStr">
-        <is>
-          <t>Technician - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C186" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Technician role</t>
-        </is>
-      </c>
-      <c r="E186" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F186" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="187" ht="120" customHeight="1">
-      <c r="A187" s="6" t="inlineStr">
-        <is>
-          <t>DI-067</t>
-        </is>
-      </c>
-      <c r="B187" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C187" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D187" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E187" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (has Create/Edit) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F187" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188" ht="135" customHeight="1">
-      <c r="A188" s="6" t="inlineStr">
-        <is>
-          <t>DI-068</t>
-        </is>
-      </c>
-      <c r="B188" s="2" t="inlineStr">
-        <is>
-          <t>Parts Manager - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C188" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D188" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The three-dot menu shows Add Inspection.
-Step 4: The inspection template is added and "Inspection added to line." is shown.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E188" s="2" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; the line three-dot menu "Add Inspection" action is available (gated by this permission), so an inspection template can be added ("Inspection added to line.").</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=Y. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="189" ht="120" customHeight="1">
-      <c r="A189" s="6" t="inlineStr">
-        <is>
-          <t>DI-070</t>
-        </is>
-      </c>
-      <c r="B189" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C189" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D189" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection opens.
-Step 3: Inspection items can be filled/edited (provided the line is not marked complete).
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E189" s="3" t="inlineStr">
-        <is>
-          <t>Role has workOrderLinesCreateAndEdit -&gt; an in-progress inspection opens and items are editable (provided the line is not marked complete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F189" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=Y (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190" ht="90" customHeight="1">
-      <c r="A190" s="6" t="inlineStr">
-        <is>
-          <t>DI-073</t>
-        </is>
-      </c>
-      <c r="B190" s="2" t="inlineStr">
-        <is>
-          <t>Parts Manager - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C190" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D190" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E190" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="191" ht="120" customHeight="1">
-      <c r="A191" s="6" t="inlineStr">
-        <is>
-          <t>DI-074</t>
-        </is>
-      </c>
-      <c r="B191" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C191" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D191" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing an inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E191" s="3" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available - role lacks workOrderLinesDelete (Work Order Lines: Delete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F191" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192" ht="120" customHeight="1">
-      <c r="A192" s="6" t="inlineStr">
-        <is>
-          <t>DI-075</t>
-        </is>
-      </c>
-      <c r="B192" s="2" t="inlineStr">
-        <is>
-          <t>Parts Manager - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C192" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D192" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E192" s="2" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available for a completed inspection - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F192" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="193" ht="120" customHeight="1">
-      <c r="A193" s="6" t="inlineStr">
-        <is>
-          <t>DI-076</t>
-        </is>
-      </c>
-      <c r="B193" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C193" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D193" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Reopen is NOT available - reopening a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E193" s="3" t="inlineStr">
-        <is>
-          <t>Reopen is NOT available - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F193" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="194" ht="255" customHeight="1">
-      <c r="A194" s="6" t="inlineStr">
-        <is>
-          <t>DI-077</t>
-        </is>
-      </c>
-      <c r="B194" s="2" t="inlineStr">
-        <is>
-          <t>Parts Manager - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C194" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Parts Manager role</t>
-        </is>
-      </c>
-      <c r="E194" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="195" ht="120" customHeight="1">
-      <c r="A195" s="6" t="inlineStr">
-        <is>
-          <t>DI-078</t>
-        </is>
-      </c>
-      <c r="B195" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C195" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D195" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E195" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (view-only) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F195" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="196" ht="135" customHeight="1">
-      <c r="A196" s="6" t="inlineStr">
-        <is>
-          <t>DI-079</t>
-        </is>
-      </c>
-      <c r="B196" s="2" t="inlineStr">
-        <is>
-          <t>Parts Technician - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C196" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Add Inspection is NOT available - role lacks Work Order Lines: Create and Edit.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E196" s="2" t="inlineStr">
-        <is>
-          <t>Add Inspection is NOT available - role lacks workOrderLinesCreateAndEdit (Work Order Lines: Create and Edit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=N. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="197" ht="90" customHeight="1">
-      <c r="A197" s="6" t="inlineStr">
-        <is>
-          <t>DI-080</t>
-        </is>
-      </c>
-      <c r="B197" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C197" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D197" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot add inspections (no Work Order Lines: Create and Edit).
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E197" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot add inspections (lacks workOrderLinesCreateAndEdit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F197" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="198" ht="120" customHeight="1">
-      <c r="A198" s="6" t="inlineStr">
-        <is>
-          <t>DI-081</t>
-        </is>
-      </c>
-      <c r="B198" s="2" t="inlineStr">
-        <is>
-          <t>Parts Technician - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C198" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection can be opened to VIEW only.
-Step 3: Items cannot be filled or edited - role lacks Work Order Lines: Create and Edit (read-only).
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E198" s="2" t="inlineStr">
-        <is>
-          <t>Inspection opens to VIEW only; items cannot be edited - role lacks workOrderLinesCreateAndEdit (read-only), matching expected.</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="199" ht="90" customHeight="1">
-      <c r="A199" s="6" t="inlineStr">
-        <is>
-          <t>DI-082</t>
-        </is>
-      </c>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C199" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot fill/submit an inspection (no Work Order Lines: Create and Edit).
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E199" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot fill/submit an inspection (lacks workOrderLinesCreateAndEdit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F199" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="200" ht="90" customHeight="1">
-      <c r="A200" s="6" t="inlineStr">
-        <is>
-          <t>DI-083</t>
-        </is>
-      </c>
-      <c r="B200" s="2" t="inlineStr">
-        <is>
-          <t>Parts Technician - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C200" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot fill an inspection. If such a state exists (set by another role), this role would only observe it as "Open".
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E200" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot fill an inspection; if such a state exists (set by another role) this role would only observe it as "Open", matching expected.</t>
-        </is>
-      </c>
-      <c r="F200" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="201" ht="90" customHeight="1">
-      <c r="A201" s="6" t="inlineStr">
-        <is>
-          <t>DI-084</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D201" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E201" s="3" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F201" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="202" ht="120" customHeight="1">
-      <c r="A202" s="6" t="inlineStr">
-        <is>
-          <t>DI-085</t>
-        </is>
-      </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>Parts Technician - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C202" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing an inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E202" s="2" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available - role lacks workOrderLinesDelete (Work Order Lines: Delete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="203" ht="120" customHeight="1">
-      <c r="A203" s="6" t="inlineStr">
-        <is>
-          <t>DI-086</t>
-        </is>
-      </c>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D203" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E203" s="3" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available for a completed inspection - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F203" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="204" ht="120" customHeight="1">
-      <c r="A204" s="6" t="inlineStr">
-        <is>
-          <t>DI-087</t>
-        </is>
-      </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>Parts Technician - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C204" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Reopen is NOT available - reopening a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E204" s="2" t="inlineStr">
-        <is>
-          <t>Reopen is NOT available - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F204" s="2" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="205" ht="255" customHeight="1">
-      <c r="A205" s="6" t="inlineStr">
-        <is>
-          <t>DI-088</t>
-        </is>
-      </c>
-      <c r="B205" s="3" t="inlineStr">
-        <is>
-          <t>Parts Technician - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C205" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D205" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Parts Technician role</t>
-        </is>
-      </c>
-      <c r="E205" s="3" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible via Settings &gt; Service - the Service settings section is not shown (role lacks settingsService), matching expected.</t>
-        </is>
-      </c>
-      <c r="F205" s="3" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role lacks settingsService so the Service menu group / Inspection Templates link is not exposed. NOTE (hardening finding): the /administration/inspection-templates route itself lacks a settingsService guard, so roles that have another settings sub-permission (e.g. Service Manager, Parts Manager) can reach a READ-ONLY view via direct URL (no "New" button); the documented Settings&gt;Service menu path is correctly denied. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="206" ht="105" customHeight="1">
-      <c r="A206" s="6" t="inlineStr">
-        <is>
-          <t>DI-089</t>
-        </is>
-      </c>
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>Office - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C206" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work order opens.
-Step 3: Existing inspections on the line are visible. Edit controls (Add/bin/Open) appear only if the role has the relevant Work Order Lines rights; otherwise the inspection is read-only.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable (verified); existing inspections on a line are visible. Edit controls (Add/bin/Open) present only per the role's Work Order Lines rights (view-only) - matches expected.</t>
-        </is>
-      </c>
-      <c r="F206" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="207" ht="135" customHeight="1">
-      <c r="A207" s="6" t="inlineStr">
-        <is>
-          <t>DI-090</t>
-        </is>
-      </c>
-      <c r="B207" s="3" t="inlineStr">
-        <is>
-          <t>Office - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C207" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D207" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Add Inspection is NOT available - role lacks Work Order Lines: Create and Edit.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E207" s="3" t="inlineStr">
-        <is>
-          <t>Add Inspection is NOT available - role lacks workOrderLinesCreateAndEdit (Work Order Lines: Create and Edit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F207" s="3" t="inlineStr">
-        <is>
-          <t>Line-level control gating verified via authoritative effective permission workOrderLinesCreateAndEdit=N. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" ht="90" customHeight="1">
-      <c r="A208" s="6" t="inlineStr">
-        <is>
-          <t>DI-091</t>
-        </is>
-      </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>Office - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C208" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D208" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot add inspections (no Work Order Lines: Create and Edit).
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E208" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot add inspections (lacks workOrderLinesCreateAndEdit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F208" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="209" ht="120" customHeight="1">
-      <c r="A209" s="6" t="inlineStr">
-        <is>
-          <t>DI-092</t>
-        </is>
-      </c>
-      <c r="B209" s="3" t="inlineStr">
-        <is>
-          <t>Office - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C209" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D209" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: The inspection can be opened to VIEW only.
-Step 3: Items cannot be filled or edited - role lacks Work Order Lines: Create and Edit (read-only).
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E209" s="3" t="inlineStr">
-        <is>
-          <t>Inspection opens to VIEW only; items cannot be edited - role lacks workOrderLinesCreateAndEdit (read-only), matching expected.</t>
-        </is>
-      </c>
-      <c r="F209" s="3" t="inlineStr">
-        <is>
-          <t>Edit-capability gated by workOrderLinesCreateAndEdit=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="210" ht="90" customHeight="1">
-      <c r="A210" s="6" t="inlineStr">
-        <is>
-          <t>DI-093</t>
-        </is>
-      </c>
-      <c r="B210" s="2" t="inlineStr">
-        <is>
-          <t>Office - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C210" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D210" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot fill/submit an inspection (no Work Order Lines: Create and Edit).
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E210" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot fill/submit an inspection (lacks workOrderLinesCreateAndEdit), matching expected.</t>
-        </is>
-      </c>
-      <c r="F210" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="211" ht="90" customHeight="1">
-      <c r="A211" s="6" t="inlineStr">
-        <is>
-          <t>DI-094</t>
-        </is>
-      </c>
-      <c r="B211" s="3" t="inlineStr">
-        <is>
-          <t>Office - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C211" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D211" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - role cannot fill an inspection. If such a state exists (set by another role), this role would only observe it as "Open".
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E211" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable - role cannot fill an inspection; if such a state exists (set by another role) this role would only observe it as "Open", matching expected.</t>
-        </is>
-      </c>
-      <c r="F211" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="212" ht="90" customHeight="1">
-      <c r="A212" s="6" t="inlineStr">
-        <is>
-          <t>DI-095</t>
-        </is>
-      </c>
-      <c r="B212" s="2" t="inlineStr">
-        <is>
-          <t>Office - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C212" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D212" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: A completed inspection shows "Completed"; an in-progress inspection shows "In Progress" with a percentage of completion.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E212" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders reachable; inspection status labels render (Completed / In Progress with percentage) - feature present and WO access confirmed, matching expected.</t>
-        </is>
-      </c>
-      <c r="F212" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="213" ht="120" customHeight="1">
-      <c r="A213" s="6" t="inlineStr">
-        <is>
-          <t>DI-096</t>
-        </is>
-      </c>
-      <c r="B213" s="3" t="inlineStr">
-        <is>
-          <t>Office - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C213" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D213" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing an inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E213" s="3" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available - role lacks workOrderLinesDelete (Work Order Lines: Delete), matching expected.</t>
-        </is>
-      </c>
-      <c r="F213" s="3" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="214" ht="120" customHeight="1">
-      <c r="A214" s="6" t="inlineStr">
-        <is>
-          <t>DI-097</t>
-        </is>
-      </c>
-      <c r="B214" s="2" t="inlineStr">
-        <is>
-          <t>Office - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C214" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D214" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: The remove (bin) control is NOT available - removing a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E214" s="2" t="inlineStr">
-        <is>
-          <t>The remove (bin) control is NOT available for a completed inspection - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>Remove control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="215" ht="120" customHeight="1">
-      <c r="A215" s="6" t="inlineStr">
-        <is>
-          <t>DI-098</t>
-        </is>
-      </c>
-      <c r="B215" s="3" t="inlineStr">
-        <is>
-          <t>Office - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C215" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D215" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Reopen is NOT available - reopening a completed inspection requires Work Order Lines: Delete.
-Spec reference: SV-7509 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E215" s="3" t="inlineStr">
-        <is>
-          <t>Reopen is NOT available - role lacks workOrderLinesDelete, matching expected.</t>
-        </is>
-      </c>
-      <c r="F215" s="3" t="inlineStr">
-        <is>
-          <t>Reopen control gated by workOrderLinesDelete=N (verified). Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="216" ht="120" customHeight="1">
-      <c r="A216" s="6" t="inlineStr">
-        <is>
-          <t>DI-099</t>
-        </is>
-      </c>
-      <c r="B216" s="2" t="inlineStr">
-        <is>
-          <t>Office - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C216" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Office" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D216" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Settings &gt; Service is accessible.
-Step 3: The Inspection Templates section is available.
-Step 4: A new template can be created with fields: Checklist, Short Text, Long Text, Measurements, Photo, Instructions.
-Spec reference: SV-7521 · Digital Inspections — Office role</t>
-        </is>
-      </c>
-      <c r="E216" s="2" t="inlineStr">
-        <is>
-          <t>Settings &gt; Service is accessible and the Service section exposes "Inspection Templates" (verified in Tech UI: SERVICE menu group shown, page loads with template list + "New/Create" control). A template can be created with the listed field types.</t>
-        </is>
-      </c>
-      <c r="F216" s="2" t="inlineStr">
-        <is>
-          <t>Requires settingsApp + settingsService; role has both. Verified live in Tech UI. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="217" ht="135" customHeight="1">
-      <c r="A217" s="6" t="inlineStr">
-        <is>
-          <t>DI-100</t>
-        </is>
-      </c>
-      <c r="B217" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C217" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D217" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work Orders are not accessible to this role.
-Step 3: Inspections cannot be reached - no Work Orders access.
-Spec reference: SV-7506 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E217" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F217" s="3" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="218" ht="135" customHeight="1">
-      <c r="A218" s="6" t="inlineStr">
-        <is>
-          <t>DI-101</t>
-        </is>
-      </c>
-      <c r="B218" s="2" t="inlineStr">
-        <is>
-          <t>Sales Representative - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C218" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D218" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access, the line cannot be reached.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E218" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F218" s="2" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="219" ht="135" customHeight="1">
-      <c r="A219" s="6" t="inlineStr">
-        <is>
-          <t>DI-102</t>
-        </is>
-      </c>
-      <c r="B219" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C219" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D219" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E219" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F219" s="3" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="220" ht="135" customHeight="1">
-      <c r="A220" s="6" t="inlineStr">
-        <is>
-          <t>DI-103</t>
-        </is>
-      </c>
-      <c r="B220" s="2" t="inlineStr">
-        <is>
-          <t>Sales Representative - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C220" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D220" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E220" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F220" s="2" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="221" ht="135" customHeight="1">
-      <c r="A221" s="6" t="inlineStr">
-        <is>
-          <t>DI-104</t>
-        </is>
-      </c>
-      <c r="B221" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C221" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D221" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E221" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F221" s="3" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="222" ht="135" customHeight="1">
-      <c r="A222" s="6" t="inlineStr">
-        <is>
-          <t>DI-105</t>
-        </is>
-      </c>
-      <c r="B222" s="2" t="inlineStr">
-        <is>
-          <t>Sales Representative - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C222" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D222" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E222" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F222" s="2" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="223" ht="135" customHeight="1">
-      <c r="A223" s="6" t="inlineStr">
-        <is>
-          <t>DI-106</t>
-        </is>
-      </c>
-      <c r="B223" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C223" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D223" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access, statuses cannot be seen.
-Spec reference: SV-7506 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E223" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F223" s="3" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="224" ht="135" customHeight="1">
-      <c r="A224" s="6" t="inlineStr">
-        <is>
-          <t>DI-107</t>
-        </is>
-      </c>
-      <c r="B224" s="2" t="inlineStr">
-        <is>
-          <t>Sales Representative - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C224" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D224" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E224" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F224" s="2" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="225" ht="135" customHeight="1">
-      <c r="A225" s="6" t="inlineStr">
-        <is>
-          <t>DI-108</t>
-        </is>
-      </c>
-      <c r="B225" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C225" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D225" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E225" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F225" s="3" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="226" ht="135" customHeight="1">
-      <c r="A226" s="6" t="inlineStr">
-        <is>
-          <t>DI-109</t>
-        </is>
-      </c>
-      <c r="B226" s="2" t="inlineStr">
-        <is>
-          <t>Sales Representative - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C226" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E226" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed no Work Orders access (role lacks workOrdersView/CreateAndEdit; Tech UI redirected away from /workorders to Reports). Inspections/lines cannot be reached - matches expected N/A.</t>
-        </is>
-      </c>
-      <c r="F226" s="2" t="inlineStr">
-        <is>
-          <t>WO-access gate = (workOrdersView OR workOrdersCreateAndEdit) + default workplace; role has neither. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="227" ht="90" customHeight="1">
-      <c r="A227" s="6" t="inlineStr">
-        <is>
-          <t>DI-110</t>
-        </is>
-      </c>
-      <c r="B227" s="3" t="inlineStr">
-        <is>
-          <t>Sales Representative - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C227" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Sales Representative" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D227" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Sales Representative role</t>
-        </is>
-      </c>
-      <c r="E227" s="3" t="inlineStr">
-        <is>
-          <t>Inspection Templates NOT accessible - role lacks settingsApp/settingsService (no Administration settings access).</t>
-        </is>
-      </c>
-      <c r="F227" s="3" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="228" ht="135" customHeight="1">
-      <c r="A228" s="6" t="inlineStr">
-        <is>
-          <t>DI-112</t>
-        </is>
-      </c>
-      <c r="B228" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - B. Add inspection to a work order line</t>
-        </is>
-      </c>
-      <c r="C228" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D228" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access, the line cannot be reached.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E228" s="2" t="inlineStr">
-        <is>
-          <t>DI action unavailable to Time Clock as required (role lacks the necessary workOrderLines permission), so the described inability holds. Note: WO itself IS reachable (has workOrdersView), unlike the "no WO access" premise.</t>
-        </is>
-      </c>
-      <c r="F228" s="2" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock has WO access via workOrdersView; DI action still correctly gated off by missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="229" ht="165" customHeight="1">
-      <c r="A229" s="6" t="inlineStr">
-        <is>
-          <t>DI-113</t>
-        </is>
-      </c>
-      <c r="B229" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C229" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D229" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E229" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable in effect - Time Clock cannot add/fill/submit an inspection (role lacks workOrderLinesCreateAndEdit). Outcome (cannot perform) matches expected, though note WO is actually reachable.</t>
-        </is>
-      </c>
-      <c r="F229" s="3" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock DOES have WO access (workOrdersView), contradicting the precondition's "no WO access"; however the inspection action is still correctly unavailable due to missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="230" ht="135" customHeight="1">
-      <c r="A230" s="6" t="inlineStr">
-        <is>
-          <t>DI-114</t>
-        </is>
-      </c>
-      <c r="B230" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - D. Open and fill an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C230" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D230" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E230" s="2" t="inlineStr">
-        <is>
-          <t>DI action unavailable to Time Clock as required (role lacks the necessary workOrderLines permission), so the described inability holds. Note: WO itself IS reachable (has workOrdersView), unlike the "no WO access" premise.</t>
-        </is>
-      </c>
-      <c r="F230" s="2" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock has WO access via workOrdersView; DI action still correctly gated off by missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="231" ht="165" customHeight="1">
-      <c r="A231" s="6" t="inlineStr">
-        <is>
-          <t>DI-115</t>
-        </is>
-      </c>
-      <c r="B231" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C231" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D231" s="3" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E231" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable in effect - Time Clock cannot add/fill/submit an inspection (role lacks workOrderLinesCreateAndEdit). Outcome (cannot perform) matches expected, though note WO is actually reachable.</t>
-        </is>
-      </c>
-      <c r="F231" s="3" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock DOES have WO access (workOrdersView), contradicting the precondition's "no WO access"; however the inspection action is still correctly unavailable due to missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="232" ht="165" customHeight="1">
-      <c r="A232" s="6" t="inlineStr">
-        <is>
-          <t>DI-116</t>
-        </is>
-      </c>
-      <c r="B232" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C232" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D232" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E232" s="2" t="inlineStr">
-        <is>
-          <t>Not applicable in effect - Time Clock cannot add/fill/submit an inspection (role lacks workOrderLinesCreateAndEdit). Outcome (cannot perform) matches expected, though note WO is actually reachable.</t>
-        </is>
-      </c>
-      <c r="F232" s="2" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock DOES have WO access (workOrdersView), contradicting the precondition's "no WO access"; however the inspection action is still correctly unavailable due to missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="233" ht="135" customHeight="1">
-      <c r="A233" s="6" t="inlineStr">
-        <is>
-          <t>DI-118</t>
-        </is>
-      </c>
-      <c r="B233" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock - H. Remove an in-progress inspection</t>
-        </is>
-      </c>
-      <c r="C233" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D233" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E233" s="3" t="inlineStr">
-        <is>
-          <t>DI action unavailable to Time Clock as required (role lacks the necessary workOrderLines permission), so the described inability holds. Note: WO itself IS reachable (has workOrdersView), unlike the "no WO access" premise.</t>
-        </is>
-      </c>
-      <c r="F233" s="3" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock has WO access via workOrdersView; DI action still correctly gated off by missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="234" ht="135" customHeight="1">
-      <c r="A234" s="6" t="inlineStr">
-        <is>
-          <t>DI-119</t>
-        </is>
-      </c>
-      <c r="B234" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - I. Remove a completed inspection</t>
-        </is>
-      </c>
-      <c r="C234" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D234" s="2" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E234" s="2" t="inlineStr">
-        <is>
-          <t>DI action unavailable to Time Clock as required (role lacks the necessary workOrderLines permission), so the described inability holds. Note: WO itself IS reachable (has workOrdersView), unlike the "no WO access" premise.</t>
-        </is>
-      </c>
-      <c r="F234" s="2" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock has WO access via workOrdersView; DI action still correctly gated off by missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="235" ht="135" customHeight="1">
-      <c r="A235" s="6" t="inlineStr">
-        <is>
-          <t>DI-120</t>
-        </is>
-      </c>
-      <c r="B235" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock - J. Reopen a completed inspection</t>
-        </is>
-      </c>
-      <c r="C235" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D235" s="3" t="inlineStr">
-        <is>
-          <t>Step 3: Not applicable - no Work Orders access.
-Spec reference: SV-7509 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E235" s="3" t="inlineStr">
-        <is>
-          <t>DI action unavailable to Time Clock as required (role lacks the necessary workOrderLines permission), so the described inability holds. Note: WO itself IS reachable (has workOrdersView), unlike the "no WO access" premise.</t>
-        </is>
-      </c>
-      <c r="F235" s="3" t="inlineStr">
-        <is>
-          <t>DRIFT NOTE: Time Clock has WO access via workOrdersView; DI action still correctly gated off by missing workOrderLines permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="236" ht="90" customHeight="1">
-      <c r="A236" s="6" t="inlineStr">
-        <is>
-          <t>DI-121</t>
-        </is>
-      </c>
-      <c r="B236" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - K. Configure Inspection Templates (Settings &gt; Service)</t>
-        </is>
-      </c>
-      <c r="C236" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D236" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Inspection Templates configuration is NOT accessible - it requires Settings plus the Service sub-setting.
-Spec reference: SV-7521 · Digital Inspections — Time Clock role</t>
-        </is>
-      </c>
-      <c r="E236" s="2" t="inlineStr">
-        <is>
-          <t>Inspection Templates configuration is NOT accessible - Time Clock lacks settingsApp/settingsService so the Administration settings area and the Service &gt; Inspection Templates menu are unavailable.</t>
-        </is>
-      </c>
-      <c r="F236" s="2" t="inlineStr">
-        <is>
-          <t>Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8436,7 +5119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -8613,88 +5296,6 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="165" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>DI-111</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock - A. View inspections on a work order line</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>1. As Admin, assign a test user the "Time Clock" role.
-2. Log out and log back in as that Time Clock user (fresh login so permissions load).
-3. Look at the left navigation and try to open Work Orders / view an inspection on a work order.</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Step 1: Login succeeds.
-Step 2: Work Orders are not accessible to this role.
-Step 3: Inspections cannot be reached - no Work Orders access.
-Spec reference: SV-7506 · Digital Inspections — Time Clock role · VIU-33: The 'Time Clock' system role is clock-in/out-only and should NOT grant Work Orders access; Work Orders and Digital Inspections should be unreachable…</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Time Clock role DOES grant workOrdersView -&gt; Work Orders ARE accessible in the Tech UI (landed on /workorders, WO list rendered). Existing inspections on a line are therefore reachable/visible (read-only, since role lacks Work Order Lines rights). This CONTRADICTS the expected "no Work Orders access".</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>DRIFT FINDING: the live "Time Clock" system role includes workOrdersView (description says "Clock in/out only"), so it has WO access, unlike the spec precondition. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="135" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>DI-117</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Time Clock - G. Inspection status labels display correctly</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Time Clock" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>1. As Admin, assign a test user the "Time Clock" role.
-2. Log out, log back in as that Time Clock user.
-3. Open a Work Order that has a Digital Inspection and look at the inspection status labels.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Step 2: Not applicable - no Work Orders access, statuses cannot be seen.
-Spec reference: SV-7506 · Digital Inspections — Time Clock role · VIU-33: The 'Time Clock' system role is clock-in/out-only and should NOT grant Work Orders access; Work Orders and Digital Inspections should be unreachable…</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Work Orders ARE accessible for Time Clock (has workOrdersView), so inspection status labels CAN be seen - contradicts expected "no Work Orders access, statuses cannot be seen".</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>DRIFT FINDING: Time Clock role grants workOrdersView -&gt; WO access exists. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8706,7 +5307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9674,678 +6275,6 @@
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Permission set correctly applied &amp; hydrated; deep line-level action not automatable non-destructively here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="150" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>DI-003</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="135" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>DI-005</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Administrator - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="120" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>DI-006</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Administrator - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Administrator" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="150" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>DI-014</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="135" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>DI-016</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Service Manager - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="120" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>DI-017</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Service Manager - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="150" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>DI-025</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="135" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>DI-027</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="120" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>DI-028</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Senior Service Advisor - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Senior Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="150" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>DI-036</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="135" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>DI-038</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Service Advisor - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="120" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>DI-039</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Service Advisor - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Service Advisor" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="150" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>DI-047</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="135" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>DI-049</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Foreman - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="120" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>DI-050</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Foreman - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Foreman" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="150" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>DI-058</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Technician - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="135" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>DI-060</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>Technician - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="120" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>DI-061</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Technician - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Technician" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="150" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>DI-069</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - C. Add multiple inspection templates to one line</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have permanently changed shared test data (and the spec does not define the exact limit being checked), so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive mutation of shared staging data + spec VIU (max-per-line unspecified). Add-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="135" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>DI-071</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Parts Manager - E. Complete an inspection (Submit and Generate Report)</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Running this test would have generated a real report / changed the status of live records on the shared test site, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: destructive (generates real PDF report / status change on shared staging). Submit-capability confirmed via permission. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="120" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>DI-072</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>Parts Manager - F. Inspection at 100 percent but not submitted shows Open</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>Test role set up as an exact copy of the built-in "Parts Manager" role, assigned to a test technician account (fresh login used so the permissions load).</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Running this test would have filled in a real inspection to 100% on the shared test site, changing data other testers rely on, so it was not executed.</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Needs a safe, disposable Digital Inspections work order (or agreement that shared staging data may be changed) so the action can be performed without harming other testers' data.</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED reason: requires destructive fill of a real inspection to 100% on shared staging. Basis: effective fe-permissions verified live via Tech quick-login (match=true vs intended); DI access is governed by these existing permissions (no dedicated DI/checklist permission exists in this org). Feature presence confirmed via /api/inspection-templates.</t>
         </is>
       </c>
     </row>

</xml_diff>